<commit_message>
PROGRAMA QUE FUNCIONA PERFECTO
Hice una estructura, 3D, con distintos apoyos, distintas cargas y anduvo PERFECTO
</commit_message>
<xml_diff>
--- a/supertesteo_resultados.xlsx
+++ b/supertesteo_resultados.xlsx
@@ -7,12 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Resumen_Fuerzas_Internas" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="F_Interna_Global" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Cargas_Globales_en_nudos" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="reacciones_locales_de_empotramiento" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Vector_Nodal_Equivalente" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="f_local_Reacc_i_por_Carga" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="reacciones_de_estructura_Globales" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Desplazamientos_globales_D" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Sistema_reducido_Kll_Fl" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Cargas_Globales_en_nudos" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="reacciones_locales_de_empotramiento" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Vector_Nodal_Equivalente" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Ejes_Locales" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Matriz_Rotacion_T" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
@@ -432,25 +432,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P5"/>
+  <dimension ref="A1:O5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="23" customWidth="1" min="5" max="5"/>
-    <col width="21" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="21" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
-    <col width="25" customWidth="1" min="10" max="10"/>
-    <col width="24" customWidth="1" min="11" max="11"/>
-    <col width="24" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="23" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
+    <col width="23" customWidth="1" min="10" max="10"/>
+    <col width="21" customWidth="1" min="11" max="11"/>
+    <col width="21" customWidth="1" min="12" max="12"/>
     <col width="21" customWidth="1" min="13" max="13"/>
-    <col width="21" customWidth="1" min="14" max="14"/>
-    <col width="23" customWidth="1" min="15" max="15"/>
-    <col width="20" customWidth="1" min="16" max="16"/>
+    <col width="24" customWidth="1" min="14" max="14"/>
+    <col width="20" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -471,67 +470,62 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Longitud (cm)</t>
+          <t>Fx_i</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Fx_i (kN)</t>
+          <t>Fy_i</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Fy_i (kN)</t>
+          <t>Fz_i</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Fz_i (kN)</t>
+          <t>Mx_i</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Mx_i (kN·cm)</t>
+          <t>My_i</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>My_i (kN·cm)</t>
+          <t>Mz_i</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Mz_i (kN·cm)</t>
+          <t>Fx_f</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Fx_f (kN)</t>
+          <t>Fy_f</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Fy_f (kN)</t>
+          <t>Fz_f</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>Fz_f (kN)</t>
+          <t>Mx_f</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>Mx_f (kN·cm)</t>
+          <t>My_f</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>My_f (kN·cm)</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>Mz_f (kN·cm)</t>
+          <t>Mz_f</t>
         </is>
       </c>
     </row>
@@ -546,42 +540,39 @@
         <v>2</v>
       </c>
       <c r="D2" t="n">
-        <v>300</v>
+        <v>0.08264608928248485</v>
       </c>
       <c r="E2" t="n">
-        <v>0.1099770941905521</v>
+        <v>0.3132746458246708</v>
       </c>
       <c r="F2" t="n">
-        <v>0.1465176493074707</v>
+        <v>5.080843638685171</v>
       </c>
       <c r="G2" t="n">
-        <v>5.279055776464235</v>
+        <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>3.552713678800501e-15</v>
       </c>
       <c r="I2" t="n">
-        <v>2.664535259100376e-15</v>
+        <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>0</v>
+        <v>-0.08264608928248485</v>
       </c>
       <c r="K2" t="n">
-        <v>-0.1099770941905521</v>
+        <v>-0.3132746458246708</v>
       </c>
       <c r="L2" t="n">
-        <v>-0.1465176493074707</v>
+        <v>-5.080843638685171</v>
       </c>
       <c r="M2" t="n">
-        <v>-5.279055776464235</v>
+        <v>-93.98239374740125</v>
       </c>
       <c r="N2" t="n">
-        <v>-43.95529479224122</v>
+        <v>24.79382678474544</v>
       </c>
       <c r="O2" t="n">
-        <v>32.99312825716563</v>
-      </c>
-      <c r="P2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -596,42 +587,39 @@
         <v>4</v>
       </c>
       <c r="D3" t="n">
-        <v>300</v>
+        <v>-2.220446049250313e-16</v>
       </c>
       <c r="E3" t="n">
-        <v>4.440892098500626e-16</v>
+        <v>2.664535259100376e-15</v>
       </c>
       <c r="F3" t="n">
-        <v>-5.000000000000002</v>
+        <v>11.39111351096038</v>
       </c>
       <c r="G3" t="n">
-        <v>11.56576802356741</v>
+        <v>2.273736754432321e-13</v>
       </c>
       <c r="H3" t="n">
-        <v>375</v>
+        <v>0</v>
       </c>
       <c r="I3" t="n">
         <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>2.220446049250313e-16</v>
       </c>
       <c r="K3" t="n">
-        <v>-4.440892098500626e-16</v>
+        <v>4.999999999999997</v>
       </c>
       <c r="L3" t="n">
-        <v>1.77635683940025e-15</v>
+        <v>-11.39111351096038</v>
       </c>
       <c r="M3" t="n">
-        <v>-11.56576802356741</v>
+        <v>749.9999999999998</v>
       </c>
       <c r="N3" t="n">
-        <v>375.0000000000002</v>
+        <v>-4.263256414560601e-14</v>
       </c>
       <c r="O3" t="n">
-        <v>9.947598300641403e-14</v>
-      </c>
-      <c r="P3" t="n">
         <v>0</v>
       </c>
     </row>
@@ -646,43 +634,40 @@
         <v>5</v>
       </c>
       <c r="D4" t="n">
-        <v>200</v>
+        <v>0.08264608928241235</v>
       </c>
       <c r="E4" t="n">
-        <v>0.1099770941904298</v>
+        <v>-4.686725354175329</v>
       </c>
       <c r="F4" t="n">
-        <v>-4.85348235069253</v>
+        <v>6.471957149645529</v>
       </c>
       <c r="G4" t="n">
-        <v>1.844823800031678</v>
+        <v>-656.0176062525985</v>
       </c>
       <c r="H4" t="n">
-        <v>-456.0447052077589</v>
+        <v>-16.70946291623017</v>
       </c>
       <c r="I4" t="n">
-        <v>-5.087550610739213</v>
+        <v>-31.32746458246704</v>
       </c>
       <c r="J4" t="n">
-        <v>-14.65176493074691</v>
+        <v>-0.08264608928241235</v>
       </c>
       <c r="K4" t="n">
-        <v>-0.1099770941904298</v>
+        <v>4.686725354175329</v>
       </c>
       <c r="L4" t="n">
-        <v>4.85348235069253</v>
+        <v>-1.471957149645529</v>
       </c>
       <c r="M4" t="n">
-        <v>-6.844823800031678</v>
+        <v>-138.3738236765075</v>
       </c>
       <c r="N4" t="n">
-        <v>-412.9200547985768</v>
+        <v>16.70946291623017</v>
       </c>
       <c r="O4" t="n">
-        <v>5.087550610739213</v>
-      </c>
-      <c r="P4" t="n">
-        <v>36.64718376883285</v>
+        <v>47.85668243894946</v>
       </c>
     </row>
     <row r="5">
@@ -696,43 +681,40 @@
         <v>4</v>
       </c>
       <c r="D5" t="n">
-        <v>100</v>
+        <v>0.08264608928243433</v>
       </c>
       <c r="E5" t="n">
-        <v>0.1099770941904126</v>
+        <v>0.3132746458246718</v>
       </c>
       <c r="F5" t="n">
-        <v>0.1465176493074694</v>
+        <v>5.080843638685151</v>
       </c>
       <c r="G5" t="n">
-        <v>-4.720944223535734</v>
+        <v>93.98239374740122</v>
       </c>
       <c r="H5" t="n">
-        <v>43.95529479224121</v>
+        <v>-24.79382678474538</v>
       </c>
       <c r="I5" t="n">
-        <v>217.0068717428343</v>
+        <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>-1.4210854715202e-14</v>
+        <v>-0.08264608928243433</v>
       </c>
       <c r="K5" t="n">
-        <v>-0.1099770941904126</v>
+        <v>-0.3132746458246718</v>
       </c>
       <c r="L5" t="n">
-        <v>-0.1465176493074694</v>
+        <v>4.919156361314849</v>
       </c>
       <c r="M5" t="n">
-        <v>-5.279055776464266</v>
+        <v>-93.98239374740122</v>
       </c>
       <c r="N5" t="n">
-        <v>-43.95529479224121</v>
+        <v>16.70946291623029</v>
       </c>
       <c r="O5" t="n">
-        <v>-244.9124493892609</v>
-      </c>
-      <c r="P5" t="n">
-        <v>14.65176493074691</v>
+        <v>31.32746458246709</v>
       </c>
     </row>
   </sheetData>
@@ -746,100 +728,52 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O5"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="23" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="21" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
-    <col width="25" customWidth="1" min="9" max="9"/>
-    <col width="24" customWidth="1" min="10" max="10"/>
-    <col width="24" customWidth="1" min="11" max="11"/>
-    <col width="21" customWidth="1" min="12" max="12"/>
-    <col width="21" customWidth="1" min="13" max="13"/>
-    <col width="23" customWidth="1" min="14" max="14"/>
-    <col width="20" customWidth="1" min="15" max="15"/>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Barra ID</t>
+          <t>Nodo ID</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Nodo Inicial</t>
+          <t>Ux</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Nodo Final</t>
+          <t>Uy</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Fx_i</t>
+          <t>Uz</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Fy_i</t>
+          <t>Rx</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Fz_i</t>
+          <t>Ry</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Mx_i</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>My_i</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Mz_i</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Fx_f</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Fy_f</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>Fz_f</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Mx_f</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>My_f</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>Mz_f</t>
+          <t>Rz</t>
         </is>
       </c>
     </row>
@@ -848,46 +782,22 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>0.1099770941905521</v>
+        <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>0.1465176493074707</v>
+        <v>0.0001042972465977096</v>
       </c>
       <c r="F2" t="n">
-        <v>5.279055776464235</v>
+        <v>9.505808433179217e-05</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H2" t="n">
-        <v>2.664535259100376e-15</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J2" t="n">
-        <v>-0.1099770941905521</v>
-      </c>
-      <c r="K2" t="n">
-        <v>-0.1465176493074707</v>
-      </c>
-      <c r="L2" t="n">
-        <v>-5.279055776464235</v>
-      </c>
-      <c r="M2" t="n">
-        <v>-43.95529479224122</v>
-      </c>
-      <c r="N2" t="n">
-        <v>32.99312825716563</v>
-      </c>
-      <c r="O2" t="n">
-        <v>0</v>
+        <v>-0.000569315001876651</v>
       </c>
     </row>
     <row r="3">
@@ -895,46 +805,22 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>3</v>
+        <v>0.05084079875519081</v>
       </c>
       <c r="C3" t="n">
-        <v>4</v>
+        <v>0.05332882759397755</v>
       </c>
       <c r="D3" t="n">
-        <v>4.440892098500626e-16</v>
+        <v>-0.0007621265458027756</v>
       </c>
       <c r="E3" t="n">
-        <v>-5.000000000000002</v>
+        <v>-0.0007418827691351947</v>
       </c>
       <c r="F3" t="n">
-        <v>11.56576802356741</v>
+        <v>0.0003182918188883237</v>
       </c>
       <c r="G3" t="n">
-        <v>375</v>
-      </c>
-      <c r="H3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J3" t="n">
-        <v>-4.440892098500626e-16</v>
-      </c>
-      <c r="K3" t="n">
-        <v>1.77635683940025e-15</v>
-      </c>
-      <c r="L3" t="n">
-        <v>-11.56576802356741</v>
-      </c>
-      <c r="M3" t="n">
-        <v>375.0000000000002</v>
-      </c>
-      <c r="N3" t="n">
-        <v>9.947598300641403e-14</v>
-      </c>
-      <c r="O3" t="n">
-        <v>0</v>
+        <v>-0.000569315001876651</v>
       </c>
     </row>
     <row r="4">
@@ -942,46 +828,22 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>4</v>
+        <v>0.1430712489045995</v>
       </c>
       <c r="C4" t="n">
-        <v>5</v>
+        <v>-1.326507896862112</v>
       </c>
       <c r="D4" t="n">
-        <v>0.1099770941904298</v>
+        <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>-4.85348235069253</v>
+        <v>-0.00498285583779166</v>
       </c>
       <c r="F4" t="n">
-        <v>1.844823800031678</v>
+        <v>-0.0003074486081795761</v>
       </c>
       <c r="G4" t="n">
-        <v>-456.0447052077589</v>
-      </c>
-      <c r="H4" t="n">
-        <v>-5.087550610739213</v>
-      </c>
-      <c r="I4" t="n">
-        <v>-14.65176493074691</v>
-      </c>
-      <c r="J4" t="n">
-        <v>-0.1099770941904298</v>
-      </c>
-      <c r="K4" t="n">
-        <v>4.85348235069253</v>
-      </c>
-      <c r="L4" t="n">
-        <v>-6.844823800031678</v>
-      </c>
-      <c r="M4" t="n">
-        <v>-412.9200547985768</v>
-      </c>
-      <c r="N4" t="n">
-        <v>5.087550610739213</v>
-      </c>
-      <c r="O4" t="n">
-        <v>36.64718376883285</v>
+        <v>-0.0004752950001285505</v>
       </c>
     </row>
     <row r="5">
@@ -989,46 +851,45 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>2</v>
+        <v>0.05083666645072668</v>
       </c>
       <c r="C5" t="n">
-        <v>4</v>
+        <v>-0.0004686725354175329</v>
       </c>
       <c r="D5" t="n">
-        <v>0.1099770941904126</v>
+        <v>-0.001708667026644057</v>
       </c>
       <c r="E5" t="n">
-        <v>0.1465176493074694</v>
+        <v>-0.001606505297575576</v>
       </c>
       <c r="F5" t="n">
-        <v>-4.720944223535734</v>
+        <v>-0.0003074486081795765</v>
       </c>
       <c r="G5" t="n">
-        <v>43.95529479224121</v>
-      </c>
-      <c r="H5" t="n">
-        <v>217.0068717428343</v>
-      </c>
-      <c r="I5" t="n">
-        <v>-1.4210854715202e-14</v>
-      </c>
-      <c r="J5" t="n">
-        <v>-0.1099770941904126</v>
-      </c>
-      <c r="K5" t="n">
-        <v>-0.1465176493074694</v>
-      </c>
-      <c r="L5" t="n">
-        <v>-5.279055776464266</v>
-      </c>
-      <c r="M5" t="n">
-        <v>-43.95529479224121</v>
-      </c>
-      <c r="N5" t="n">
-        <v>-244.9124493892609</v>
-      </c>
-      <c r="O5" t="n">
-        <v>14.65176493074691</v>
+        <v>-0.0004752950001285505</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1037,6 +898,1516 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:V21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="21" customWidth="1" min="12" max="12"/>
+    <col width="21" customWidth="1" min="13" max="13"/>
+    <col width="21" customWidth="1" min="14" max="14"/>
+    <col width="20" customWidth="1" min="15" max="15"/>
+    <col width="21" customWidth="1" min="16" max="16"/>
+    <col width="21" customWidth="1" min="17" max="17"/>
+    <col width="21" customWidth="1" min="18" max="18"/>
+    <col width="21" customWidth="1" min="19" max="19"/>
+    <col width="21" customWidth="1" min="20" max="20"/>
+    <col width="20" customWidth="1" min="21" max="21"/>
+    <col width="8" customWidth="1" min="22" max="22"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>DOF_global_fila</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>K_dof_3</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>K_dof_4</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>K_dof_5</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>K_dof_6</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>K_dof_7</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>K_dof_8</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>K_dof_9</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>K_dof_10</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>K_dof_11</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>K_dof_12</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>K_dof_13</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>K_dof_15</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>K_dof_16</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>K_dof_17</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>K_dof_18</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>K_dof_19</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>K_dof_20</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>K_dof_21</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>K_dof_22</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>K_dof_23</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>Fl</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B2" t="n">
+        <v>222133.3333333333</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>1110.666666666667</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>111066.6666666667</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U2" t="n">
+        <v>0</v>
+      </c>
+      <c r="V2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" t="n">
+        <v>222133.3333333333</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>-1110.666666666667</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>111066.6666666667</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R3" t="n">
+        <v>0</v>
+      </c>
+      <c r="S3" t="n">
+        <v>0</v>
+      </c>
+      <c r="T3" t="n">
+        <v>0</v>
+      </c>
+      <c r="U3" t="n">
+        <v>0</v>
+      </c>
+      <c r="V3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" t="n">
+        <v>36232.53333333333</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" t="n">
+        <v>-36232.53333333333</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" t="n">
+        <v>-1110.666666666667</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>20007.40444444444</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>-1110.666666666667</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P5" t="n">
+        <v>-20000</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S5" t="n">
+        <v>0</v>
+      </c>
+      <c r="T5" t="n">
+        <v>0</v>
+      </c>
+      <c r="U5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>7</v>
+      </c>
+      <c r="B6" t="n">
+        <v>1110.666666666667</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>207.3244444444445</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>1110.666666666667</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" t="n">
+        <v>9996</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>-199.92</v>
+      </c>
+      <c r="R6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U6" t="n">
+        <v>9996</v>
+      </c>
+      <c r="V6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>8</v>
+      </c>
+      <c r="B7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>6866.586666666667</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="n">
+        <v>-9996</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>0</v>
+      </c>
+      <c r="R7" t="n">
+        <v>-199.92</v>
+      </c>
+      <c r="S7" t="n">
+        <v>0</v>
+      </c>
+      <c r="T7" t="n">
+        <v>-9996</v>
+      </c>
+      <c r="U7" t="n">
+        <v>0</v>
+      </c>
+      <c r="V7" t="n">
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>9</v>
+      </c>
+      <c r="B8" t="n">
+        <v>111066.6666666667</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1110.666666666667</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
+        <v>330830.9333333333</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" t="n">
+        <v>0</v>
+      </c>
+      <c r="P8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>0</v>
+      </c>
+      <c r="R8" t="n">
+        <v>0</v>
+      </c>
+      <c r="S8" t="n">
+        <v>-108697.6</v>
+      </c>
+      <c r="T8" t="n">
+        <v>0</v>
+      </c>
+      <c r="U8" t="n">
+        <v>0</v>
+      </c>
+      <c r="V8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>10</v>
+      </c>
+      <c r="B9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" t="n">
+        <v>111066.6666666667</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>-1110.666666666667</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
+        <v>-9996</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="n">
+        <v>888533.3333333334</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" t="n">
+        <v>0</v>
+      </c>
+      <c r="P9" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>0</v>
+      </c>
+      <c r="R9" t="n">
+        <v>9996</v>
+      </c>
+      <c r="S9" t="n">
+        <v>0</v>
+      </c>
+      <c r="T9" t="n">
+        <v>333200</v>
+      </c>
+      <c r="U9" t="n">
+        <v>0</v>
+      </c>
+      <c r="V9" t="n">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>11</v>
+      </c>
+      <c r="B10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" t="n">
+        <v>-36232.53333333333</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="n">
+        <v>9996</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" t="n">
+        <v>702632.5333333333</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0</v>
+      </c>
+      <c r="N10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>-9996</v>
+      </c>
+      <c r="R10" t="n">
+        <v>0</v>
+      </c>
+      <c r="S10" t="n">
+        <v>0</v>
+      </c>
+      <c r="T10" t="n">
+        <v>0</v>
+      </c>
+      <c r="U10" t="n">
+        <v>333200</v>
+      </c>
+      <c r="V10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>12</v>
+      </c>
+      <c r="B11" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" t="n">
+        <v>7.404444444444445</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" t="n">
+        <v>1110.666666666667</v>
+      </c>
+      <c r="O11" t="n">
+        <v>0</v>
+      </c>
+      <c r="P11" t="n">
+        <v>-7.404444444444445</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>0</v>
+      </c>
+      <c r="R11" t="n">
+        <v>0</v>
+      </c>
+      <c r="S11" t="n">
+        <v>0</v>
+      </c>
+      <c r="T11" t="n">
+        <v>1110.666666666667</v>
+      </c>
+      <c r="U11" t="n">
+        <v>0</v>
+      </c>
+      <c r="V11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>13</v>
+      </c>
+      <c r="B12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" t="n">
+        <v>7.404444444444445</v>
+      </c>
+      <c r="M12" t="n">
+        <v>-1110.666666666667</v>
+      </c>
+      <c r="N12" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" t="n">
+        <v>0</v>
+      </c>
+      <c r="P12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>-7.404444444444445</v>
+      </c>
+      <c r="R12" t="n">
+        <v>0</v>
+      </c>
+      <c r="S12" t="n">
+        <v>-1110.666666666667</v>
+      </c>
+      <c r="T12" t="n">
+        <v>0</v>
+      </c>
+      <c r="U12" t="n">
+        <v>0</v>
+      </c>
+      <c r="V12" t="n">
+        <v>-2.5</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>15</v>
+      </c>
+      <c r="B13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" t="n">
+        <v>-1110.666666666667</v>
+      </c>
+      <c r="M13" t="n">
+        <v>222133.3333333333</v>
+      </c>
+      <c r="N13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" t="n">
+        <v>0</v>
+      </c>
+      <c r="P13" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>1110.666666666667</v>
+      </c>
+      <c r="R13" t="n">
+        <v>0</v>
+      </c>
+      <c r="S13" t="n">
+        <v>111066.6666666667</v>
+      </c>
+      <c r="T13" t="n">
+        <v>0</v>
+      </c>
+      <c r="U13" t="n">
+        <v>0</v>
+      </c>
+      <c r="V13" t="n">
+        <v>187.5</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>16</v>
+      </c>
+      <c r="B14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" t="n">
+        <v>1110.666666666667</v>
+      </c>
+      <c r="L14" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" t="n">
+        <v>222133.3333333333</v>
+      </c>
+      <c r="O14" t="n">
+        <v>0</v>
+      </c>
+      <c r="P14" t="n">
+        <v>-1110.666666666667</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>0</v>
+      </c>
+      <c r="R14" t="n">
+        <v>0</v>
+      </c>
+      <c r="S14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T14" t="n">
+        <v>111066.6666666667</v>
+      </c>
+      <c r="U14" t="n">
+        <v>0</v>
+      </c>
+      <c r="V14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>17</v>
+      </c>
+      <c r="B15" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" t="n">
+        <v>36232.53333333333</v>
+      </c>
+      <c r="P15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>0</v>
+      </c>
+      <c r="R15" t="n">
+        <v>0</v>
+      </c>
+      <c r="S15" t="n">
+        <v>0</v>
+      </c>
+      <c r="T15" t="n">
+        <v>0</v>
+      </c>
+      <c r="U15" t="n">
+        <v>-36232.53333333333</v>
+      </c>
+      <c r="V15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>18</v>
+      </c>
+      <c r="B16" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" t="n">
+        <v>-20000</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" t="n">
+        <v>-7.404444444444445</v>
+      </c>
+      <c r="L16" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" t="n">
+        <v>-1110.666666666667</v>
+      </c>
+      <c r="O16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P16" t="n">
+        <v>20032.39444444445</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>0</v>
+      </c>
+      <c r="R16" t="n">
+        <v>0</v>
+      </c>
+      <c r="S16" t="n">
+        <v>0</v>
+      </c>
+      <c r="T16" t="n">
+        <v>-1110.666666666667</v>
+      </c>
+      <c r="U16" t="n">
+        <v>2499</v>
+      </c>
+      <c r="V16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>19</v>
+      </c>
+      <c r="B17" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" t="n">
+        <v>-199.92</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" t="n">
+        <v>-9996</v>
+      </c>
+      <c r="K17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" t="n">
+        <v>-7.404444444444445</v>
+      </c>
+      <c r="M17" t="n">
+        <v>1110.666666666667</v>
+      </c>
+      <c r="N17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" t="n">
+        <v>0</v>
+      </c>
+      <c r="P17" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>10207.32444444444</v>
+      </c>
+      <c r="R17" t="n">
+        <v>0</v>
+      </c>
+      <c r="S17" t="n">
+        <v>1110.666666666667</v>
+      </c>
+      <c r="T17" t="n">
+        <v>0</v>
+      </c>
+      <c r="U17" t="n">
+        <v>-9996</v>
+      </c>
+      <c r="V17" t="n">
+        <v>-2.5</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>20</v>
+      </c>
+      <c r="B18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" t="n">
+        <v>-199.92</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" t="n">
+        <v>9996</v>
+      </c>
+      <c r="J18" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" t="n">
+        <v>0</v>
+      </c>
+      <c r="M18" t="n">
+        <v>0</v>
+      </c>
+      <c r="N18" t="n">
+        <v>0</v>
+      </c>
+      <c r="O18" t="n">
+        <v>0</v>
+      </c>
+      <c r="P18" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>0</v>
+      </c>
+      <c r="R18" t="n">
+        <v>6891.576666666667</v>
+      </c>
+      <c r="S18" t="n">
+        <v>-2499</v>
+      </c>
+      <c r="T18" t="n">
+        <v>9996</v>
+      </c>
+      <c r="U18" t="n">
+        <v>0</v>
+      </c>
+      <c r="V18" t="n">
+        <v>-7.5</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>21</v>
+      </c>
+      <c r="B19" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" t="n">
+        <v>-108697.6</v>
+      </c>
+      <c r="I19" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" t="n">
+        <v>-1110.666666666667</v>
+      </c>
+      <c r="M19" t="n">
+        <v>111066.6666666667</v>
+      </c>
+      <c r="N19" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" t="n">
+        <v>0</v>
+      </c>
+      <c r="P19" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>1110.666666666667</v>
+      </c>
+      <c r="R19" t="n">
+        <v>-2499</v>
+      </c>
+      <c r="S19" t="n">
+        <v>664030.9333333333</v>
+      </c>
+      <c r="T19" t="n">
+        <v>0</v>
+      </c>
+      <c r="U19" t="n">
+        <v>0</v>
+      </c>
+      <c r="V19" t="n">
+        <v>-62.5</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>22</v>
+      </c>
+      <c r="B20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" t="n">
+        <v>-9996</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" t="n">
+        <v>333200</v>
+      </c>
+      <c r="J20" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" t="n">
+        <v>1110.666666666667</v>
+      </c>
+      <c r="L20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M20" t="n">
+        <v>0</v>
+      </c>
+      <c r="N20" t="n">
+        <v>111066.6666666667</v>
+      </c>
+      <c r="O20" t="n">
+        <v>0</v>
+      </c>
+      <c r="P20" t="n">
+        <v>-1110.666666666667</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>0</v>
+      </c>
+      <c r="R20" t="n">
+        <v>9996</v>
+      </c>
+      <c r="S20" t="n">
+        <v>0</v>
+      </c>
+      <c r="T20" t="n">
+        <v>942882.1333333333</v>
+      </c>
+      <c r="U20" t="n">
+        <v>0</v>
+      </c>
+      <c r="V20" t="n">
+        <v>-125</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>23</v>
+      </c>
+      <c r="B21" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" t="n">
+        <v>9996</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" t="n">
+        <v>0</v>
+      </c>
+      <c r="J21" t="n">
+        <v>333200</v>
+      </c>
+      <c r="K21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M21" t="n">
+        <v>0</v>
+      </c>
+      <c r="N21" t="n">
+        <v>0</v>
+      </c>
+      <c r="O21" t="n">
+        <v>-36232.53333333333</v>
+      </c>
+      <c r="P21" t="n">
+        <v>2499</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>-9996</v>
+      </c>
+      <c r="R21" t="n">
+        <v>0</v>
+      </c>
+      <c r="S21" t="n">
+        <v>0</v>
+      </c>
+      <c r="T21" t="n">
+        <v>0</v>
+      </c>
+      <c r="U21" t="n">
+        <v>1035832.533333333</v>
+      </c>
+      <c r="V21" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1332,7 +2703,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1628,7 +2999,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1795,315 +3166,6 @@
         <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:S4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="18" customWidth="1" min="12" max="12"/>
-    <col width="18" customWidth="1" min="13" max="13"/>
-    <col width="18" customWidth="1" min="14" max="14"/>
-    <col width="18" customWidth="1" min="15" max="15"/>
-    <col width="18" customWidth="1" min="16" max="16"/>
-    <col width="18" customWidth="1" min="17" max="17"/>
-    <col width="18" customWidth="1" min="18" max="18"/>
-    <col width="18" customWidth="1" min="19" max="19"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Carga ID</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Barra ID</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Nodo Inicial</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Nodo Final</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>f_local_x</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>f_local_y</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>f_local_z</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Reacc_i_Fx_local</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Reacc_i_Fy_local</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Reacc_i_Fz_local</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Reacc_i_Mx_local</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>Reacc_i_My_local</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Reacc_i_Mz_local</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>Reacc_f_Fx_local</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>Reacc_f_Fy_local</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>Reacc_f_Fz_local</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>Reacc_f_Mx_local</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>Reacc_f_My_local</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>Reacc_f_Mz_local</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B2" t="n">
-        <v>2</v>
-      </c>
-      <c r="C2" t="n">
-        <v>3</v>
-      </c>
-      <c r="D2" t="n">
-        <v>4</v>
-      </c>
-      <c r="E2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F2" t="n">
-        <v>-5</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="J2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M2" t="n">
-        <v>187.5</v>
-      </c>
-      <c r="N2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O2" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="P2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R2" t="n">
-        <v>0</v>
-      </c>
-      <c r="S2" t="n">
-        <v>-187.5</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" t="n">
-        <v>3</v>
-      </c>
-      <c r="C3" t="n">
-        <v>4</v>
-      </c>
-      <c r="D3" t="n">
-        <v>5</v>
-      </c>
-      <c r="E3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G3" t="n">
-        <v>-5</v>
-      </c>
-      <c r="H3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J3" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="K3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L3" t="n">
-        <v>-125</v>
-      </c>
-      <c r="M3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N3" t="n">
-        <v>0</v>
-      </c>
-      <c r="O3" t="n">
-        <v>0</v>
-      </c>
-      <c r="P3" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>0</v>
-      </c>
-      <c r="R3" t="n">
-        <v>125</v>
-      </c>
-      <c r="S3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" t="n">
-        <v>4</v>
-      </c>
-      <c r="C4" t="n">
-        <v>2</v>
-      </c>
-      <c r="D4" t="n">
-        <v>4</v>
-      </c>
-      <c r="E4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G4" t="n">
-        <v>-10</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J4" t="n">
-        <v>5</v>
-      </c>
-      <c r="K4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L4" t="n">
-        <v>-125</v>
-      </c>
-      <c r="M4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P4" t="n">
-        <v>5</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>0</v>
-      </c>
-      <c r="R4" t="n">
-        <v>125</v>
-      </c>
-      <c r="S4" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Esfuerzo de corte en Y hecho
verificó con el SAP2000
</commit_message>
<xml_diff>
--- a/supertesteo_resultados.xlsx
+++ b/supertesteo_resultados.xlsx
@@ -8,13 +8,14 @@
   </bookViews>
   <sheets>
     <sheet name="reacciones_de_estructura_Globales" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Desplazamientos_globales_D" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Sistema_reducido_Kll_Fl" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Cargas_Globales_en_nudos" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="reacciones_locales_de_empotramiento" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Vector_Nodal_Equivalente" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Ejes_Locales" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Matriz_Rotacion_T" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="F_interna_Locales" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Desplazamientos_globales_D" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Sistema_reducido_Kll_Fl" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Cargas_Globales_en_nudos" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="reacciones_locales_de_empotramiento" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Vector_Nodal_Equivalente" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Ejes_Locales" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Matriz_Rotacion_T" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -728,6 +729,302 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:O5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="23" customWidth="1" min="8" max="8"/>
+    <col width="25" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
+    <col width="21" customWidth="1" min="13" max="13"/>
+    <col width="24" customWidth="1" min="14" max="14"/>
+    <col width="20" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Barra ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Nodo Inicial</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Nodo Final</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Fx_i</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Fy_i</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Fz_i</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Mx_i</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>My_i</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Mz_i</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Fx_f</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Fy_f</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Fz_f</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Mx_f</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>My_f</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Mz_f</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D2" t="n">
+        <v>5.080843638685171</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.3132746458246708</v>
+      </c>
+      <c r="F2" t="n">
+        <v>-0.08264608928248485</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>3.552713678800501e-15</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="n">
+        <v>-5.080843638685171</v>
+      </c>
+      <c r="K2" t="n">
+        <v>-0.3132746458246708</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.08264608928248485</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" t="n">
+        <v>24.79382678474544</v>
+      </c>
+      <c r="O2" t="n">
+        <v>93.98239374740125</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="n">
+        <v>3</v>
+      </c>
+      <c r="C3" t="n">
+        <v>4</v>
+      </c>
+      <c r="D3" t="n">
+        <v>11.39111351096038</v>
+      </c>
+      <c r="E3" t="n">
+        <v>2.664535259100376e-15</v>
+      </c>
+      <c r="F3" t="n">
+        <v>2.220446049250313e-16</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>-2.273736754432321e-13</v>
+      </c>
+      <c r="J3" t="n">
+        <v>-11.39111351096038</v>
+      </c>
+      <c r="K3" t="n">
+        <v>4.999999999999997</v>
+      </c>
+      <c r="L3" t="n">
+        <v>-2.220446049250313e-16</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" t="n">
+        <v>-4.263256414560601e-14</v>
+      </c>
+      <c r="O3" t="n">
+        <v>-749.9999999999998</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="n">
+        <v>4</v>
+      </c>
+      <c r="C4" t="n">
+        <v>5</v>
+      </c>
+      <c r="D4" t="n">
+        <v>4.686725354175329</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.08264608928241235</v>
+      </c>
+      <c r="F4" t="n">
+        <v>6.471957149645529</v>
+      </c>
+      <c r="G4" t="n">
+        <v>16.70946291623017</v>
+      </c>
+      <c r="H4" t="n">
+        <v>-656.0176062525985</v>
+      </c>
+      <c r="I4" t="n">
+        <v>-31.32746458246704</v>
+      </c>
+      <c r="J4" t="n">
+        <v>-4.686725354175329</v>
+      </c>
+      <c r="K4" t="n">
+        <v>-0.08264608928241235</v>
+      </c>
+      <c r="L4" t="n">
+        <v>-1.471957149645529</v>
+      </c>
+      <c r="M4" t="n">
+        <v>-16.70946291623017</v>
+      </c>
+      <c r="N4" t="n">
+        <v>-138.3738236765075</v>
+      </c>
+      <c r="O4" t="n">
+        <v>47.85668243894946</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.08264608928243433</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.3132746458246718</v>
+      </c>
+      <c r="F5" t="n">
+        <v>5.080843638685151</v>
+      </c>
+      <c r="G5" t="n">
+        <v>93.98239374740122</v>
+      </c>
+      <c r="H5" t="n">
+        <v>-24.79382678474538</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" t="n">
+        <v>-0.08264608928243433</v>
+      </c>
+      <c r="K5" t="n">
+        <v>-0.3132746458246718</v>
+      </c>
+      <c r="L5" t="n">
+        <v>4.919156361314849</v>
+      </c>
+      <c r="M5" t="n">
+        <v>-93.98239374740122</v>
+      </c>
+      <c r="N5" t="n">
+        <v>16.70946291623029</v>
+      </c>
+      <c r="O5" t="n">
+        <v>31.32746458246709</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -897,7 +1194,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2407,7 +2704,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2703,7 +3000,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2999,7 +3296,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3174,7 +3471,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3452,7 +3749,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>